<commit_message>
Added components for the sorption toolbox
</commit_message>
<xml_diff>
--- a/data/components.xlsx
+++ b/data/components.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cverhoosel/Documents/2_Education/4CBLA30_Energy_Storage_and_Transport/Energy-Storage-and-Transport.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D465BD-1559-A740-9897-3E5F7517EC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF3A52A-84CA-E649-AA1A-FED537543782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" xr2:uid="{B795D2B2-84D1-4D57-9EC8-769A1489C68E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21920" xr2:uid="{B795D2B2-84D1-4D57-9EC8-769A1489C68E}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="201">
   <si>
     <t>Name</t>
   </si>
@@ -472,9 +472,6 @@
     <t>EST-G0003</t>
   </si>
   <si>
-    <t>load cell (DCjack to terminal)</t>
-  </si>
-  <si>
     <t>EST-G0004</t>
   </si>
   <si>
@@ -535,12 +532,6 @@
     <t>EST-T0005</t>
   </si>
   <si>
-    <t>Temperature Sensor Connector (jack to Screw-Terminal)</t>
-  </si>
-  <si>
-    <t>(diagram,DS18B20_Connector_Diagram.png)</t>
-  </si>
-  <si>
     <t>EST-T0006</t>
   </si>
   <si>
@@ -590,6 +581,66 @@
   </si>
   <si>
     <t>kleinpvc tankje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power Supply TCM 24V </t>
+  </si>
+  <si>
+    <t>24V 8A DC</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>EST-E0006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHT22 RHT </t>
+  </si>
+  <si>
+    <t>EST-S0009</t>
+  </si>
+  <si>
+    <t>Heater Unit For TCM</t>
+  </si>
+  <si>
+    <t>Silica Reactor</t>
+  </si>
+  <si>
+    <t>Load Cell up to 1kg</t>
+  </si>
+  <si>
+    <t>120W Heater with PMD2406PTV1AU fan and integrated 2x DHT22</t>
+  </si>
+  <si>
+    <t>Including Bottom and Top Sepperator, DHT22 Sensor, and attachment for Loadcell</t>
+  </si>
+  <si>
+    <t>Heater Controller 24V for TCM</t>
+  </si>
+  <si>
+    <t>Including INA226 Voltage and Current Sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load cell </t>
+  </si>
+  <si>
+    <t>Load Cell (DCjack to terminal)??</t>
+  </si>
+  <si>
+    <t>Temperature and RH Sensor Connector (jack to Screw-Terminal)</t>
+  </si>
+  <si>
+    <t>DHT22 RHT Sensor, already mounted on TCM setup</t>
+  </si>
+  <si>
+    <t>Sorption</t>
+  </si>
+  <si>
+    <t>(diagram,DS18B20_Connector_Diagram.png);(diagram,DHT22_Connector_Diagram.png)</t>
+  </si>
+  <si>
+    <t>(specs,https://elektronicavoorjou.nl/product/dht22-temp-vocht-sensor/)</t>
   </si>
 </sst>
 </file>
@@ -688,7 +739,17 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color auto="1"/>
@@ -752,9 +813,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7DC69B98-0BD3-6F4A-8A7B-E3E9EDB4ADF1}" name="Table1" displayName="Table1" ref="A1:N60" totalsRowShown="0">
-  <autoFilter ref="A1:N60" xr:uid="{7DC69B98-0BD3-6F4A-8A7B-E3E9EDB4ADF1}"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7DC69B98-0BD3-6F4A-8A7B-E3E9EDB4ADF1}" name="Table1" displayName="Table1" ref="A1:O66" totalsRowShown="0">
+  <autoFilter ref="A1:O66" xr:uid="{7DC69B98-0BD3-6F4A-8A7B-E3E9EDB4ADF1}"/>
+  <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{E99DB23D-5EA5-5245-8B4B-981E39D03E25}" name="Name"/>
     <tableColumn id="2" xr3:uid="{8239B4C0-BCF3-0445-B10A-C84239A2EF89}" name="Description"/>
     <tableColumn id="3" xr3:uid="{D9F5B246-2D06-544D-8256-2199C40940D8}" name="Links"/>
@@ -773,6 +834,7 @@
     <tableColumn id="12" xr3:uid="{050F5F9F-B42D-A44F-BB9B-AF9E69C2982C}" name="Pneumatic "/>
     <tableColumn id="13" xr3:uid="{01BEC54C-FD3D-F149-A748-779377CB2494}" name="Hydraulic"/>
     <tableColumn id="14" xr3:uid="{8CE6A97A-BD80-8D41-8DBD-148DA15B09C4}" name="Thermal"/>
+    <tableColumn id="15" xr3:uid="{C7A315C7-2644-4EB8-B7C6-30650AB9552B}" name="Sorption"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1095,18 +1157,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3983C56F-212F-4EB6-9B74-522C3257755A}">
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.5" customWidth="1"/>
+    <col min="3" max="3" width="59.33203125" customWidth="1"/>
     <col min="4" max="4" width="9.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -1116,7 +1178,7 @@
     <col min="20" max="20" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1159,8 +1221,11 @@
       <c r="N1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1171,7 +1236,7 @@
         <v>16</v>
       </c>
       <c r="H2">
-        <f t="shared" ref="H2:H43" si="0">G2-J2-I2</f>
+        <f t="shared" ref="H2:H7" si="0">G2-J2-I2</f>
         <v>0</v>
       </c>
       <c r="I2">
@@ -1179,7 +1244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1203,11 +1268,11 @@
       </c>
       <c r="H3">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I3">
-        <f>K3*Toolboxes!B$1+L3*Toolboxes!B$2+M3*Toolboxes!B$3+N3*Toolboxes!B$4</f>
-        <v>80</v>
+        <f>K3*Toolboxes!B$1+L3*Toolboxes!B$2+M3*Toolboxes!B$3+N3*Toolboxes!B$4+O3*Toolboxes!B$5</f>
+        <v>90</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -1221,8 +1286,11 @@
       <c r="N3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1244,7 +1312,7 @@
         <v>47</v>
       </c>
       <c r="I4">
-        <f>K4*Toolboxes!B$1+L4*Toolboxes!B$2+M4*Toolboxes!B$3+N4*Toolboxes!B$4</f>
+        <f>K4*Toolboxes!B$1+L4*Toolboxes!B$2+M4*Toolboxes!B$3+N4*Toolboxes!B$4+O4*Toolboxes!B$5</f>
         <v>60</v>
       </c>
       <c r="K4">
@@ -1257,7 +1325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1278,18 +1346,18 @@
         <v>21</v>
       </c>
       <c r="H5">
-        <f t="shared" si="0"/>
+        <f>G5-J5-I5</f>
         <v>1</v>
       </c>
       <c r="I5">
-        <f>K5*Toolboxes!B$1+L5*Toolboxes!B$2+M5*Toolboxes!B$3+N5*Toolboxes!B$4</f>
+        <f>K5*Toolboxes!B$1+L5*Toolboxes!B$2+M5*Toolboxes!B$3+N5*Toolboxes!B$4+O5*Toolboxes!B$5</f>
         <v>20</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -1304,1353 +1372,1528 @@
         <v>-1</v>
       </c>
       <c r="I6">
-        <f>K6*Toolboxes!B$1+L6*Toolboxes!B$2+M6*Toolboxes!B$3+N6*Toolboxes!B$4</f>
+        <f>K6*Toolboxes!B$1+L6*Toolboxes!B$2+M6*Toolboxes!B$3+N6*Toolboxes!B$4+O6*Toolboxes!B$5</f>
         <v>20</v>
       </c>
       <c r="N6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
+        <v>182</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>183</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>184</v>
       </c>
       <c r="G7">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>40</v>
-      </c>
-      <c r="N7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+        <f>K7*Toolboxes!B$1+L7*Toolboxes!B$2+M7*Toolboxes!B$3+N7*Toolboxes!B$4+O7*Toolboxes!B$5</f>
+        <v>10</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
+        <v>33</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
         <v>21</v>
       </c>
       <c r="F8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8">
+        <v>18</v>
+      </c>
+      <c r="H8">
+        <f t="shared" ref="H8:H45" si="1">G8-J8-I8</f>
+        <v>-22</v>
+      </c>
+      <c r="I8">
+        <f>K8*Toolboxes!B$1+L8*Toolboxes!B$2+M8*Toolboxes!B$3+N8*Toolboxes!B$4+O8*Toolboxes!B$5</f>
+        <v>40</v>
+      </c>
+      <c r="N8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B9" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" t="s">
+        <v>200</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>186</v>
+      </c>
+      <c r="G9">
+        <v>30</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <f>K9*Toolboxes!B$1+L9*Toolboxes!B$2+M9*Toolboxes!B$3+N9*Toolboxes!B$4+O9*Toolboxes!B$5</f>
+        <v>30</v>
+      </c>
+      <c r="O9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
         <v>39</v>
       </c>
-      <c r="G8">
+      <c r="G10">
         <f xml:space="preserve"> 20 + 12</f>
         <v>32</v>
       </c>
-      <c r="H8">
-        <f t="shared" si="0"/>
+      <c r="H10">
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="I8">
-        <f>K8*Toolboxes!B$1+L8*Toolboxes!B$2+M8*Toolboxes!B$3+N8*Toolboxes!B$4</f>
+      <c r="I10">
+        <f>K10*Toolboxes!B$1+L10*Toolboxes!B$2+M10*Toolboxes!B$3+N10*Toolboxes!B$4+O10*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="M8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>40</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C11" t="s">
         <v>42</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F11" t="s">
         <v>43</v>
       </c>
-      <c r="H9">
-        <f t="shared" si="0"/>
+      <c r="H11">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I9">
-        <f>K9*Toolboxes!B$1+L9*Toolboxes!B$2+M9*Toolboxes!B$3+N9*Toolboxes!B$4</f>
+      <c r="I11">
+        <f>K11*Toolboxes!B$1+L11*Toolboxes!B$2+M11*Toolboxes!B$3+N11*Toolboxes!B$4+O11*Toolboxes!B$5</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>44</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B12" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C12" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D12" t="s">
         <v>20</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E12" t="s">
         <v>47</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F12" t="s">
         <v>48</v>
       </c>
-      <c r="G10">
+      <c r="G12">
         <v>5</v>
       </c>
-      <c r="H10">
-        <f t="shared" si="0"/>
+      <c r="H12">
+        <f t="shared" si="1"/>
         <v>-15</v>
       </c>
-      <c r="I10">
-        <f>K10*Toolboxes!B$1+L10*Toolboxes!B$2+M10*Toolboxes!B$3+N10*Toolboxes!B$4</f>
+      <c r="I12">
+        <f>K12*Toolboxes!B$1+L12*Toolboxes!B$2+M12*Toolboxes!B$3+N12*Toolboxes!B$4+O12*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="L12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E13" t="s">
         <v>47</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F13" t="s">
         <v>51</v>
       </c>
-      <c r="G11">
+      <c r="G13">
         <f xml:space="preserve"> 40+1</f>
         <v>41</v>
       </c>
-      <c r="H11">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="I11">
-        <f>K11*Toolboxes!B$1+L11*Toolboxes!B$2+M11*Toolboxes!B$3+N11*Toolboxes!B$4</f>
+      <c r="H13">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <f>K13*Toolboxes!B$1+L13*Toolboxes!B$2+M13*Toolboxes!B$3+N13*Toolboxes!B$4+O13*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L11">
+      <c r="L13">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C14" t="s">
         <v>53</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D14" t="s">
         <v>20</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E14" t="s">
         <v>21</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F14" t="s">
         <v>54</v>
       </c>
-      <c r="G12">
+      <c r="G14">
         <f>20+1</f>
         <v>21</v>
       </c>
-      <c r="H12">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="I12">
-        <f>K12*Toolboxes!B$1+L12*Toolboxes!B$2+M12*Toolboxes!B$3+N12*Toolboxes!B$4</f>
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <f>K14*Toolboxes!B$1+L14*Toolboxes!B$2+M14*Toolboxes!B$3+N14*Toolboxes!B$4+O14*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="K12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="K14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>55</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C15" t="s">
         <v>56</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D15" t="s">
         <v>20</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E15" t="s">
         <v>21</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F15" t="s">
         <v>57</v>
       </c>
-      <c r="G13">
+      <c r="G15">
         <v>24</v>
       </c>
-      <c r="H13">
-        <f t="shared" si="0"/>
+      <c r="H15">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="I13">
-        <f>K13*Toolboxes!B$1+L13*Toolboxes!B$2+M13*Toolboxes!B$3+N13*Toolboxes!B$4</f>
+      <c r="I15">
+        <f>K15*Toolboxes!B$1+L15*Toolboxes!B$2+M15*Toolboxes!B$3+N15*Toolboxes!B$4+O15*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="K13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="K15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>58</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C16" t="s">
         <v>59</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D16" t="s">
         <v>20</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E16" t="s">
         <v>21</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F16" t="s">
         <v>60</v>
       </c>
-      <c r="G14">
+      <c r="G16">
         <v>45</v>
       </c>
-      <c r="H14">
-        <f t="shared" si="0"/>
+      <c r="H16">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="I14">
+      <c r="I16">
+        <f>K16*Toolboxes!B$1+L16*Toolboxes!B$2+M16*Toolboxes!B$3+N16*Toolboxes!B$4+O16*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="K14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="K16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>61</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E17" t="s">
         <v>47</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F17" t="s">
         <v>62</v>
       </c>
-      <c r="G15">
+      <c r="G17">
         <f>40+28</f>
         <v>68</v>
       </c>
-      <c r="H15">
-        <f t="shared" si="0"/>
+      <c r="H17">
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="I15">
-        <f>K15*Toolboxes!B$1+L15*Toolboxes!B$2+M15*Toolboxes!B$3+N15*Toolboxes!B$4</f>
+      <c r="I17">
+        <f>K17*Toolboxes!B$1+L17*Toolboxes!B$2+M17*Toolboxes!B$3+N17*Toolboxes!B$4+O17*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>63</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E18" t="s">
         <v>47</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F18" t="s">
         <v>64</v>
       </c>
-      <c r="G16">
+      <c r="G18">
         <f>40+38</f>
         <v>78</v>
       </c>
-      <c r="H16">
-        <f t="shared" si="0"/>
+      <c r="H18">
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
-      <c r="I16">
-        <f>K16*Toolboxes!B$1+L16*Toolboxes!B$2+M16*Toolboxes!B$3+N16*Toolboxes!B$4</f>
+      <c r="I18">
+        <f>K18*Toolboxes!B$1+L18*Toolboxes!B$2+M18*Toolboxes!B$3+N18*Toolboxes!B$4+O18*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>65</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E19" t="s">
         <v>47</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F19" t="s">
         <v>66</v>
       </c>
-      <c r="G17">
+      <c r="G19">
         <f>40+32</f>
         <v>72</v>
       </c>
-      <c r="H17">
-        <f t="shared" si="0"/>
+      <c r="H19">
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
-      <c r="I17">
-        <f>K17*Toolboxes!B$1+L17*Toolboxes!B$2+M17*Toolboxes!B$3+N17*Toolboxes!B$4</f>
+      <c r="I19">
+        <f>K19*Toolboxes!B$1+L19*Toolboxes!B$2+M19*Toolboxes!B$3+N19*Toolboxes!B$4+O19*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L17">
+      <c r="L19">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>67</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E20" t="s">
         <v>47</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F20" t="s">
         <v>68</v>
       </c>
-      <c r="G18">
+      <c r="G20">
         <f>20+16</f>
         <v>36</v>
       </c>
-      <c r="H18">
-        <f t="shared" si="0"/>
+      <c r="H20">
+        <f t="shared" si="1"/>
         <v>-44</v>
       </c>
-      <c r="I18">
-        <f>K18*Toolboxes!B$1+L18*Toolboxes!B$2+M18*Toolboxes!B$3+N18*Toolboxes!B$4</f>
+      <c r="I20">
+        <f>K20*Toolboxes!B$1+L20*Toolboxes!B$2+M20*Toolboxes!B$3+N20*Toolboxes!B$4+O20*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L18">
+      <c r="L20">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>69</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E21" t="s">
         <v>47</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F21" t="s">
         <v>70</v>
       </c>
-      <c r="G19">
+      <c r="G21">
         <f>80+29</f>
         <v>109</v>
       </c>
-      <c r="H19">
-        <f t="shared" si="0"/>
+      <c r="H21">
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="I19">
-        <f>K19*Toolboxes!B$1+L19*Toolboxes!B$2+M19*Toolboxes!B$3+N19*Toolboxes!B$4</f>
+      <c r="I21">
+        <f>K21*Toolboxes!B$1+L21*Toolboxes!B$2+M21*Toolboxes!B$3+N21*Toolboxes!B$4+O21*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L19">
+      <c r="L21">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>71</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E22" t="s">
         <v>47</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F22" t="s">
         <v>72</v>
       </c>
-      <c r="G20">
+      <c r="G22">
         <f>40+18</f>
         <v>58</v>
       </c>
-      <c r="H20">
-        <f t="shared" si="0"/>
+      <c r="H22">
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="I20">
-        <f>K20*Toolboxes!B$1+L20*Toolboxes!B$2+M20*Toolboxes!B$3+N20*Toolboxes!B$4</f>
+      <c r="I22">
+        <f>K22*Toolboxes!B$1+L22*Toolboxes!B$2+M22*Toolboxes!B$3+N22*Toolboxes!B$4+O22*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L20">
+      <c r="L22">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>73</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E23" t="s">
         <v>47</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F23" t="s">
         <v>74</v>
       </c>
-      <c r="G21">
+      <c r="G23">
         <f>40+11</f>
         <v>51</v>
       </c>
-      <c r="H21">
-        <f t="shared" si="0"/>
+      <c r="H23">
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="I21">
-        <f>K21*Toolboxes!B$1+L21*Toolboxes!B$2+M21*Toolboxes!B$3+N21*Toolboxes!B$4</f>
+      <c r="I23">
+        <f>K23*Toolboxes!B$1+L23*Toolboxes!B$2+M23*Toolboxes!B$3+N23*Toolboxes!B$4+O23*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L21">
+      <c r="L23">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>75</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E24" t="s">
         <v>47</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F24" t="s">
         <v>76</v>
       </c>
-      <c r="G22">
+      <c r="G24">
         <f>40+10</f>
         <v>50</v>
       </c>
-      <c r="H22">
-        <f t="shared" si="0"/>
+      <c r="H24">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="I22">
-        <f>K22*Toolboxes!B$1+L22*Toolboxes!B$2+M22*Toolboxes!B$3+N22*Toolboxes!B$4</f>
+      <c r="I24">
+        <f>K24*Toolboxes!B$1+L24*Toolboxes!B$2+M24*Toolboxes!B$3+N24*Toolboxes!B$4+O24*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L22">
+      <c r="L24">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>77</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E25" t="s">
         <v>47</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F25" t="s">
         <v>78</v>
       </c>
-      <c r="G23">
+      <c r="G25">
         <f>80+2</f>
         <v>82</v>
       </c>
-      <c r="H23">
-        <f t="shared" si="0"/>
+      <c r="H25">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="I23">
-        <f>K23*Toolboxes!B$1+L23*Toolboxes!B$2+M23*Toolboxes!B$3+N23*Toolboxes!B$4</f>
+      <c r="I25">
+        <f>K25*Toolboxes!B$1+L25*Toolboxes!B$2+M25*Toolboxes!B$3+N25*Toolboxes!B$4+O25*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L23">
+      <c r="L25">
         <v>2</v>
       </c>
-      <c r="M23">
+      <c r="M25">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>79</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E26" t="s">
         <v>47</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F26" t="s">
         <v>80</v>
       </c>
-      <c r="G24">
+      <c r="G26">
         <f>80+24</f>
         <v>104</v>
       </c>
-      <c r="H24">
-        <f t="shared" si="0"/>
+      <c r="H26">
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="I24">
-        <f>K24*Toolboxes!B$1+L24*Toolboxes!B$2+M24*Toolboxes!B$3+N24*Toolboxes!B$4</f>
+      <c r="I26">
+        <f>K26*Toolboxes!B$1+L26*Toolboxes!B$2+M26*Toolboxes!B$3+N26*Toolboxes!B$4+O26*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L24">
+      <c r="L26">
         <v>2</v>
       </c>
-      <c r="M24">
+      <c r="M26">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>81</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E27" t="s">
         <v>47</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F27" t="s">
         <v>82</v>
       </c>
-      <c r="G25">
+      <c r="G27">
         <f>80+8</f>
         <v>88</v>
       </c>
-      <c r="H25">
-        <f t="shared" si="0"/>
+      <c r="H27">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="I25">
-        <f>K25*Toolboxes!B$1+L25*Toolboxes!B$2+M25*Toolboxes!B$3+N25*Toolboxes!B$4</f>
+      <c r="I27">
+        <f>K27*Toolboxes!B$1+L27*Toolboxes!B$2+M27*Toolboxes!B$3+N27*Toolboxes!B$4+O27*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L25">
+      <c r="L27">
         <v>2</v>
       </c>
-      <c r="M25">
+      <c r="M27">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>83</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E28" t="s">
         <v>47</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F28" t="s">
         <v>84</v>
       </c>
-      <c r="G26">
+      <c r="G28">
         <f>100+12</f>
         <v>112</v>
       </c>
-      <c r="H26">
-        <f t="shared" si="0"/>
+      <c r="H28">
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
-      <c r="I26">
-        <f>K26*Toolboxes!B$1+L26*Toolboxes!B$2+M26*Toolboxes!B$3+N26*Toolboxes!B$4</f>
+      <c r="I28">
+        <f>K28*Toolboxes!B$1+L28*Toolboxes!B$2+M28*Toolboxes!B$3+N28*Toolboxes!B$4+O28*Toolboxes!B$5</f>
         <v>60</v>
       </c>
-      <c r="L26">
+      <c r="L28">
         <v>2</v>
       </c>
-      <c r="M26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="M28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>85</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E29" t="s">
         <v>47</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F29" t="s">
         <v>86</v>
       </c>
-      <c r="G27">
+      <c r="G29">
         <f>80+22</f>
         <v>102</v>
       </c>
-      <c r="H27">
-        <f t="shared" si="0"/>
+      <c r="H29">
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="I27">
-        <f>K27*Toolboxes!B$1+L27*Toolboxes!B$2+M27*Toolboxes!B$3+N27*Toolboxes!B$4</f>
+      <c r="I29">
+        <f>K29*Toolboxes!B$1+L29*Toolboxes!B$2+M29*Toolboxes!B$3+N29*Toolboxes!B$4+O29*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L27">
+      <c r="L29">
         <v>2</v>
       </c>
-      <c r="M27">
+      <c r="M29">
         <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>87</v>
-      </c>
-      <c r="E28" t="s">
-        <v>88</v>
-      </c>
-      <c r="F28" t="s">
-        <v>89</v>
-      </c>
-      <c r="H28">
-        <f t="shared" si="0"/>
-        <v>-40</v>
-      </c>
-      <c r="I28">
-        <v>40</v>
-      </c>
-      <c r="L28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>90</v>
-      </c>
-      <c r="E29" t="s">
-        <v>88</v>
-      </c>
-      <c r="F29" t="s">
-        <v>91</v>
-      </c>
-      <c r="H29">
-        <f t="shared" si="0"/>
-        <v>-40</v>
-      </c>
-      <c r="I29">
-        <v>40</v>
-      </c>
-      <c r="L29">
-        <v>1</v>
-      </c>
-      <c r="M29">
-        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" t="s">
+        <v>88</v>
+      </c>
+      <c r="F30" t="s">
+        <v>89</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="1"/>
+        <v>-40</v>
+      </c>
+      <c r="I30">
+        <f>K30*Toolboxes!B$1+L30*Toolboxes!B$2+M30*Toolboxes!B$3+N30*Toolboxes!B$4+O30*Toolboxes!B$5</f>
+        <v>40</v>
+      </c>
+      <c r="L30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" t="s">
+        <v>91</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="1"/>
+        <v>-40</v>
+      </c>
+      <c r="I31">
+        <f>K31*Toolboxes!B$1+L31*Toolboxes!B$2+M31*Toolboxes!B$3+N31*Toolboxes!B$4+O31*Toolboxes!B$5</f>
+        <v>40</v>
+      </c>
+      <c r="L31">
+        <v>1</v>
+      </c>
+      <c r="M31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>92</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E32" t="s">
         <v>47</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F32" t="s">
         <v>93</v>
       </c>
-      <c r="G30">
+      <c r="G32">
         <f>80+35</f>
         <v>115</v>
       </c>
-      <c r="H30">
-        <f t="shared" si="0"/>
+      <c r="H32">
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
-      <c r="I30">
-        <f>K30*Toolboxes!B$1+L30*Toolboxes!B$2+M30*Toolboxes!B$3+N30*Toolboxes!B$4</f>
+      <c r="I32">
+        <f>K32*Toolboxes!B$1+L32*Toolboxes!B$2+M32*Toolboxes!B$3+N32*Toolboxes!B$4+O32*Toolboxes!B$5</f>
         <v>80</v>
       </c>
-      <c r="L30">
+      <c r="L32">
         <v>2</v>
       </c>
-      <c r="M30">
+      <c r="M32">
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>94</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E33" t="s">
         <v>95</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F33" t="s">
         <v>96</v>
       </c>
-      <c r="G31">
+      <c r="G33">
         <f xml:space="preserve"> 40 + 4</f>
         <v>44</v>
       </c>
-      <c r="H31">
-        <f t="shared" si="0"/>
+      <c r="H33">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="I31">
-        <f>K31*Toolboxes!B$1+L31*Toolboxes!B$2+M31*Toolboxes!B$3+N31*Toolboxes!B$4</f>
+      <c r="I33">
+        <f>K33*Toolboxes!B$1+L33*Toolboxes!B$2+M33*Toolboxes!B$3+N33*Toolboxes!B$4+O33*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L31">
-        <v>1</v>
-      </c>
-      <c r="M31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>97</v>
-      </c>
-      <c r="E32" t="s">
-        <v>47</v>
-      </c>
-      <c r="F32" t="s">
-        <v>98</v>
-      </c>
-      <c r="H32">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I32">
-        <f>K32*Toolboxes!B$1+L32*Toolboxes!B$2+M32*Toolboxes!B$3+N32*Toolboxes!B$4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>99</v>
-      </c>
-      <c r="E33" t="s">
-        <v>47</v>
-      </c>
-      <c r="F33" t="s">
-        <v>100</v>
-      </c>
-      <c r="H33">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I33">
-        <f>K33*Toolboxes!B$1+L33*Toolboxes!B$2+M33*Toolboxes!B$3+N33*Toolboxes!B$4</f>
-        <v>0</v>
+      <c r="L33">
+        <v>1</v>
+      </c>
+      <c r="M33">
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E34" t="s">
         <v>47</v>
       </c>
       <c r="F34" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I34">
-        <f>K34*Toolboxes!B$1+L34*Toolboxes!B$2+M34*Toolboxes!B$3+N34*Toolboxes!B$4</f>
+        <f>K34*Toolboxes!B$1+L34*Toolboxes!B$2+M34*Toolboxes!B$3+N34*Toolboxes!B$4+O34*Toolboxes!B$5</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>103</v>
-      </c>
-      <c r="B35" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E35" t="s">
         <v>47</v>
       </c>
       <c r="F35" t="s">
+        <v>100</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <f>K35*Toolboxes!B$1+L35*Toolboxes!B$2+M35*Toolboxes!B$3+N35*Toolboxes!B$4+O35*Toolboxes!B$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>101</v>
+      </c>
+      <c r="E36" t="s">
+        <v>47</v>
+      </c>
+      <c r="F36" t="s">
+        <v>102</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <f>K36*Toolboxes!B$1+L36*Toolboxes!B$2+M36*Toolboxes!B$3+N36*Toolboxes!B$4+O36*Toolboxes!B$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" t="s">
+        <v>104</v>
+      </c>
+      <c r="E37" t="s">
+        <v>47</v>
+      </c>
+      <c r="F37" t="s">
         <v>105</v>
       </c>
-      <c r="G35">
+      <c r="G37">
         <f xml:space="preserve"> 20 + 16</f>
         <v>36</v>
       </c>
-      <c r="H35">
-        <f t="shared" si="0"/>
+      <c r="H37">
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="I35">
-        <f>K35*Toolboxes!B$1+L35*Toolboxes!B$2+M35*Toolboxes!B$3+N35*Toolboxes!B$4</f>
+      <c r="I37">
+        <f>K37*Toolboxes!B$1+L37*Toolboxes!B$2+M37*Toolboxes!B$3+N37*Toolboxes!B$4+O37*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="L35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="L37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>106</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B38" t="s">
         <v>107</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E38" t="s">
         <v>47</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F38" t="s">
         <v>108</v>
       </c>
-      <c r="G36">
+      <c r="G38">
         <v>34</v>
       </c>
-      <c r="H36">
-        <f t="shared" si="0"/>
+      <c r="H38">
+        <f t="shared" si="1"/>
         <v>-6</v>
       </c>
-      <c r="I36">
-        <f>K36*Toolboxes!B$1+L36*Toolboxes!B$2+M36*Toolboxes!B$3+N36*Toolboxes!B$4</f>
+      <c r="I38">
+        <f>K38*Toolboxes!B$1+L38*Toolboxes!B$2+M38*Toolboxes!B$3+N38*Toolboxes!B$4+O38*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L36">
+      <c r="L38">
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>109</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B39" t="s">
         <v>110</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E39" t="s">
         <v>47</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F39" t="s">
         <v>111</v>
       </c>
-      <c r="G37">
+      <c r="G39">
         <f xml:space="preserve"> 40 + 6</f>
         <v>46</v>
       </c>
-      <c r="H37">
-        <f t="shared" si="0"/>
+      <c r="H39">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="I37">
-        <f>K37*Toolboxes!B$1+L37*Toolboxes!B$2+M37*Toolboxes!B$3+N37*Toolboxes!B$4</f>
+      <c r="I39">
+        <f>K39*Toolboxes!B$1+L39*Toolboxes!B$2+M39*Toolboxes!B$3+N39*Toolboxes!B$4+O39*Toolboxes!B$5</f>
         <v>40</v>
       </c>
-      <c r="L37">
+      <c r="L39">
         <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>112</v>
-      </c>
-      <c r="F38" t="s">
-        <v>113</v>
-      </c>
-      <c r="G38">
-        <v>2</v>
-      </c>
-      <c r="H38">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="I38">
-        <f>K38*Toolboxes!B$1+L38*Toolboxes!B$2+M38*Toolboxes!B$3+N38*Toolboxes!B$4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>114</v>
-      </c>
-      <c r="B39" t="s">
-        <v>115</v>
-      </c>
-      <c r="E39" t="s">
-        <v>116</v>
-      </c>
-      <c r="F39" t="s">
-        <v>117</v>
-      </c>
-      <c r="G39">
-        <v>25</v>
-      </c>
-      <c r="H39">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="I39">
-        <f>K39*Toolboxes!B$1+L39*Toolboxes!B$2+M39*Toolboxes!B$3+N39*Toolboxes!B$4</f>
-        <v>20</v>
-      </c>
-      <c r="M39">
-        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>112</v>
+      </c>
+      <c r="F40" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40">
+        <v>2</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="I40">
+        <f>K40*Toolboxes!B$1+L40*Toolboxes!B$2+M40*Toolboxes!B$3+N40*Toolboxes!B$4+O40*Toolboxes!B$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" t="s">
+        <v>115</v>
+      </c>
+      <c r="E41" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" t="s">
+        <v>117</v>
+      </c>
+      <c r="G41">
+        <v>25</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="I41">
+        <f>K41*Toolboxes!B$1+L41*Toolboxes!B$2+M41*Toolboxes!B$3+N41*Toolboxes!B$4+O41*Toolboxes!B$5</f>
+        <v>20</v>
+      </c>
+      <c r="M41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>118</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B42" t="s">
         <v>119</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F42" t="s">
         <v>120</v>
       </c>
-      <c r="G40">
+      <c r="G42">
         <f>20+8</f>
         <v>28</v>
       </c>
-      <c r="H40">
-        <f t="shared" si="0"/>
+      <c r="H42">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="I40">
+      <c r="I42">
+        <f>K42*Toolboxes!B$1+L42*Toolboxes!B$2+M42*Toolboxes!B$3+N42*Toolboxes!B$4+O42*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="M40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="M42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
         <v>121</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F43" t="s">
         <v>122</v>
       </c>
-      <c r="G41">
+      <c r="G43">
         <f>20+13</f>
         <v>33</v>
       </c>
-      <c r="H41">
-        <f t="shared" si="0"/>
+      <c r="H43">
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="I41">
+      <c r="I43">
+        <f>K43*Toolboxes!B$1+L43*Toolboxes!B$2+M43*Toolboxes!B$3+N43*Toolboxes!B$4+O43*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="M41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
+      <c r="M43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B42" s="1"/>
-      <c r="E42" t="s">
+      <c r="B44" s="1"/>
+      <c r="E44" t="s">
         <v>116</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F44" t="s">
         <v>124</v>
       </c>
-      <c r="G42">
+      <c r="G44">
         <v>21</v>
       </c>
-      <c r="H42">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="I42">
+      <c r="H44">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="I44">
+        <f>K44*Toolboxes!B$1+L44*Toolboxes!B$2+M44*Toolboxes!B$3+N44*Toolboxes!B$4+O44*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="M42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>125</v>
-      </c>
-      <c r="F43" t="s">
-        <v>126</v>
-      </c>
-      <c r="H43">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I43">
-        <f>K43*Toolboxes!B$1+L43*Toolboxes!B$2+M43*Toolboxes!B$3+N43*Toolboxes!B$4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>127</v>
-      </c>
-      <c r="F44" t="s">
-        <v>128</v>
-      </c>
-      <c r="G44">
-        <v>1</v>
-      </c>
-      <c r="H44">
-        <f t="shared" ref="H44" si="1">G44-J44-I44</f>
-        <v>0</v>
-      </c>
-      <c r="I44">
+      <c r="M44">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F45" t="s">
-        <v>130</v>
-      </c>
-      <c r="G45">
-        <v>20</v>
+        <v>126</v>
       </c>
       <c r="H45">
-        <f>G45-J45-I45</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I45">
-        <v>20</v>
+        <f>K45*Toolboxes!B$1+L45*Toolboxes!B$2+M45*Toolboxes!B$3+N45*Toolboxes!B$4+O45*Toolboxes!B$5</f>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="F46" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G46">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H46">
-        <f>G46-J46-I46</f>
-        <v>5</v>
+        <f t="shared" ref="H46" si="2">G46-J46-I46</f>
+        <v>1</v>
       </c>
       <c r="I46">
-        <f>K46*Toolboxes!B$1+L46*Toolboxes!B$2+M46*Toolboxes!B$3+N46*Toolboxes!B$4</f>
+        <f>K46*Toolboxes!B$1+L46*Toolboxes!B$2+M46*Toolboxes!B$3+N46*Toolboxes!B$4+O46*Toolboxes!B$5</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>133</v>
-      </c>
-      <c r="B47" t="s">
-        <v>134</v>
-      </c>
-      <c r="C47" t="s">
-        <v>135</v>
-      </c>
-      <c r="D47" t="s">
-        <v>28</v>
-      </c>
-      <c r="E47" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="F47" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="G47">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H47">
         <f>G47-J47-I47</f>
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I47">
-        <f>K47*Toolboxes!B$1+L47*Toolboxes!B$2+M47*Toolboxes!B$3+N47*Toolboxes!B$4</f>
-        <v>20</v>
-      </c>
-      <c r="K47">
-        <v>1</v>
+        <f>K47*Toolboxes!B$1+L47*Toolboxes!B$2+M47*Toolboxes!B$3+N47*Toolboxes!B$4+O47*Toolboxes!B$5</f>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>138</v>
-      </c>
-      <c r="E48" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="F48" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="G48">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="H48">
         <f>G48-J48-I48</f>
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I48">
-        <f>K48*Toolboxes!B$1+L48*Toolboxes!B$2+M48*Toolboxes!B$3+N48*Toolboxes!B$4</f>
-        <v>20</v>
-      </c>
-      <c r="K48">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+        <f>K48*Toolboxes!B$1+L48*Toolboxes!B$2+M48*Toolboxes!B$3+N48*Toolboxes!B$4+O48*Toolboxes!B$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B49" t="s">
-        <v>141</v>
+        <v>134</v>
+      </c>
+      <c r="C49" t="s">
+        <v>135</v>
+      </c>
+      <c r="D49" t="s">
+        <v>28</v>
       </c>
       <c r="E49" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F49" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G49">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H49">
         <f>G49-J49-I49</f>
+        <v>4</v>
+      </c>
+      <c r="I49">
+        <f>K49*Toolboxes!B$1+L49*Toolboxes!B$2+M49*Toolboxes!B$3+N49*Toolboxes!B$4+O49*Toolboxes!B$5</f>
+        <v>20</v>
+      </c>
+      <c r="K49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>138</v>
+      </c>
+      <c r="E50" t="s">
+        <v>116</v>
+      </c>
+      <c r="F50" t="s">
+        <v>139</v>
+      </c>
+      <c r="G50">
+        <v>45</v>
+      </c>
+      <c r="H50">
+        <f>G50-J50-I50</f>
+        <v>25</v>
+      </c>
+      <c r="I50">
+        <f>K50*Toolboxes!B$1+L50*Toolboxes!B$2+M50*Toolboxes!B$3+N50*Toolboxes!B$4+O50*Toolboxes!B$5</f>
+        <v>20</v>
+      </c>
+      <c r="K50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>140</v>
+      </c>
+      <c r="B51" t="s">
+        <v>141</v>
+      </c>
+      <c r="E51" t="s">
+        <v>142</v>
+      </c>
+      <c r="F51" t="s">
+        <v>143</v>
+      </c>
+      <c r="G51">
+        <v>22</v>
+      </c>
+      <c r="H51">
+        <f>G51-J51-I51</f>
         <v>2</v>
       </c>
-      <c r="I49">
-        <f>K49*Toolboxes!B$1+L49*Toolboxes!B$2+M49*Toolboxes!B$3+N49*Toolboxes!B$4</f>
+      <c r="I51">
+        <f>K51*Toolboxes!B$1+L51*Toolboxes!B$2+M51*Toolboxes!B$3+N51*Toolboxes!B$4+O51*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="K49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="K51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>195</v>
+      </c>
+      <c r="F52" t="s">
         <v>144</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G52">
+        <v>30</v>
+      </c>
+      <c r="H52">
+        <f t="shared" ref="H52:H53" si="3">G52-J52-I52</f>
+        <v>30</v>
+      </c>
+      <c r="I52">
+        <f>K52*Toolboxes!B$1+L52*Toolboxes!B$2+M52*Toolboxes!B$3+N52*Toolboxes!B$4+O52*Toolboxes!B$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>145</v>
       </c>
-      <c r="G50">
-        <f xml:space="preserve"> 20 + 10</f>
-        <v>30</v>
-      </c>
-      <c r="H50">
-        <f t="shared" ref="H50:H51" si="2">G50-J50-I50</f>
-        <v>10</v>
-      </c>
-      <c r="I50">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="F53" t="s">
         <v>146</v>
       </c>
-      <c r="F51" t="s">
-        <v>147</v>
-      </c>
-      <c r="G51">
+      <c r="G53">
         <v>21</v>
-      </c>
-      <c r="H51">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="I51">
-        <v>20</v>
-      </c>
-      <c r="K51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>148</v>
-      </c>
-      <c r="B52" t="s">
-        <v>149</v>
-      </c>
-      <c r="F52" t="s">
-        <v>150</v>
-      </c>
-      <c r="H52">
-        <f t="shared" ref="H52:H60" si="3">G52-J52-I52</f>
-        <v>0</v>
-      </c>
-      <c r="I52">
-        <f>K52*Toolboxes!B$1+L52*Toolboxes!B$2+M52*Toolboxes!B$3+N52*Toolboxes!B$4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>151</v>
-      </c>
-      <c r="B53" t="s">
-        <v>152</v>
-      </c>
-      <c r="F53" t="s">
-        <v>153</v>
       </c>
       <c r="H53">
         <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="I53">
+        <f>K53*Toolboxes!B$1+L53*Toolboxes!B$2+M53*Toolboxes!B$3+N53*Toolboxes!B$4+O53*Toolboxes!B$5</f>
+        <v>20</v>
+      </c>
+      <c r="K53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>147</v>
+      </c>
+      <c r="B54" t="s">
+        <v>148</v>
+      </c>
+      <c r="F54" t="s">
+        <v>149</v>
+      </c>
+      <c r="H54">
+        <f t="shared" ref="H54:H63" si="4">G54-J54-I54</f>
         <v>0</v>
       </c>
-      <c r="I53">
-        <f>K53*Toolboxes!B$1+L53*Toolboxes!B$2+M53*Toolboxes!B$3+N53*Toolboxes!B$4</f>
+      <c r="I54">
+        <f>K54*Toolboxes!B$1+L54*Toolboxes!B$2+M54*Toolboxes!B$3+N54*Toolboxes!B$4+O54*Toolboxes!B$5</f>
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B55" t="s">
+        <v>151</v>
+      </c>
+      <c r="F55" t="s">
+        <v>152</v>
+      </c>
+      <c r="H55">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <f>K55*Toolboxes!B$1+L55*Toolboxes!B$2+M55*Toolboxes!B$3+N55*Toolboxes!B$4+O55*Toolboxes!B$5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>153</v>
+      </c>
+      <c r="B56" t="s">
         <v>154</v>
       </c>
-      <c r="B54" t="s">
+      <c r="F56" t="s">
         <v>155</v>
       </c>
-      <c r="F54" t="s">
+      <c r="H56">
+        <f t="shared" si="4"/>
+        <v>-20</v>
+      </c>
+      <c r="I56">
+        <f>K56*Toolboxes!B$1+L56*Toolboxes!B$2+M56*Toolboxes!B$3+N56*Toolboxes!B$4+O56*Toolboxes!B$5</f>
+        <v>20</v>
+      </c>
+      <c r="N56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>156</v>
       </c>
-      <c r="H54">
-        <f t="shared" si="3"/>
+      <c r="F57" t="s">
+        <v>157</v>
+      </c>
+      <c r="H57">
+        <f t="shared" si="4"/>
         <v>-20</v>
       </c>
-      <c r="I54">
-        <f>K54*Toolboxes!B$1+L54*Toolboxes!B$2+M54*Toolboxes!B$3+N54*Toolboxes!B$4</f>
+      <c r="I57">
+        <f>K57*Toolboxes!B$1+L57*Toolboxes!B$2+M57*Toolboxes!B$3+N57*Toolboxes!B$4+O57*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="N54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>157</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="N57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>158</v>
       </c>
-      <c r="H55">
-        <f t="shared" si="3"/>
+      <c r="F58" t="s">
+        <v>159</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="4"/>
         <v>-20</v>
       </c>
-      <c r="I55">
-        <f>K55*Toolboxes!B$1+L55*Toolboxes!B$2+M55*Toolboxes!B$3+N55*Toolboxes!B$4</f>
+      <c r="I58">
+        <f>K58*Toolboxes!B$1+L58*Toolboxes!B$2+M58*Toolboxes!B$3+N58*Toolboxes!B$4+O58*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="N55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>159</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="N58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>160</v>
       </c>
-      <c r="H56">
-        <f t="shared" si="3"/>
+      <c r="F59" t="s">
+        <v>161</v>
+      </c>
+      <c r="H59">
+        <f t="shared" si="4"/>
         <v>-20</v>
       </c>
-      <c r="I56">
-        <f>K56*Toolboxes!B$1+L56*Toolboxes!B$2+M56*Toolboxes!B$3+N56*Toolboxes!B$4</f>
+      <c r="I59">
+        <f>K59*Toolboxes!B$1+L59*Toolboxes!B$2+M59*Toolboxes!B$3+N59*Toolboxes!B$4+O59*Toolboxes!B$5</f>
         <v>20</v>
       </c>
-      <c r="N56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>161</v>
-      </c>
-      <c r="F57" t="s">
+      <c r="N59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
         <v>162</v>
       </c>
-      <c r="H57">
-        <f t="shared" si="3"/>
-        <v>-20</v>
-      </c>
-      <c r="I57">
-        <f>K57*Toolboxes!B$1+L57*Toolboxes!B$2+M57*Toolboxes!B$3+N57*Toolboxes!B$4</f>
-        <v>20</v>
-      </c>
-      <c r="N57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="F60" t="s">
         <v>163</v>
       </c>
-      <c r="F58" t="s">
+      <c r="H60">
+        <f t="shared" si="4"/>
+        <v>-40</v>
+      </c>
+      <c r="I60">
+        <f>K60*Toolboxes!B$1+L60*Toolboxes!B$2+M60*Toolboxes!B$3+N60*Toolboxes!B$4+O60*Toolboxes!B$5</f>
+        <v>40</v>
+      </c>
+      <c r="N60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>196</v>
+      </c>
+      <c r="C61" t="s">
+        <v>199</v>
+      </c>
+      <c r="F61" t="s">
         <v>164</v>
       </c>
-      <c r="H58">
-        <f t="shared" si="3"/>
-        <v>-40</v>
-      </c>
-      <c r="I58">
-        <f>K58*Toolboxes!B$1+L58*Toolboxes!B$2+M58*Toolboxes!B$3+N58*Toolboxes!B$4</f>
+      <c r="G61">
+        <v>100</v>
+      </c>
+      <c r="H61">
+        <f>G61-J61-I61</f>
         <v>40</v>
       </c>
-      <c r="N58">
+      <c r="I61">
+        <f>K61*Toolboxes!B$1+L61*Toolboxes!B$2+M61*Toolboxes!B$3+N61*Toolboxes!B$4+O61*Toolboxes!B$5</f>
+        <v>60</v>
+      </c>
+      <c r="N61">
         <v>2</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="O61">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>165</v>
       </c>
-      <c r="C59" t="s">
+      <c r="F62" t="s">
         <v>166</v>
       </c>
-      <c r="F59" t="s">
-        <v>167</v>
-      </c>
-      <c r="H59">
-        <f t="shared" si="3"/>
-        <v>-40</v>
-      </c>
-      <c r="I59">
-        <f>K59*Toolboxes!B$1+L59*Toolboxes!B$2+M59*Toolboxes!B$3+N59*Toolboxes!B$4</f>
-        <v>40</v>
-      </c>
-      <c r="N59">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>168</v>
-      </c>
-      <c r="F60" t="s">
-        <v>169</v>
-      </c>
-      <c r="H60">
-        <f t="shared" si="3"/>
+      <c r="H62">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I60">
-        <f>K60*Toolboxes!B$1+L60*Toolboxes!B$2+M60*Toolboxes!B$3+N60*Toolboxes!B$4</f>
+      <c r="I62">
+        <f>K62*Toolboxes!B$1+L62*Toolboxes!B$2+M62*Toolboxes!B$3+N62*Toolboxes!B$4+O62*Toolboxes!B$5</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>187</v>
+      </c>
+      <c r="B63" t="s">
+        <v>190</v>
+      </c>
+      <c r="F63" t="s">
+        <v>35</v>
+      </c>
+      <c r="G63">
+        <v>10</v>
+      </c>
+      <c r="H63">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <f>K63*Toolboxes!B$1+L63*Toolboxes!B$2+M63*Toolboxes!B$3+N63*Toolboxes!B$4+O63*Toolboxes!B$5</f>
+        <v>10</v>
+      </c>
+      <c r="O63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>188</v>
+      </c>
+      <c r="B64" t="s">
+        <v>191</v>
+      </c>
+      <c r="F64" t="s">
+        <v>39</v>
+      </c>
+      <c r="G64">
+        <v>10</v>
+      </c>
+      <c r="H64">
+        <f t="shared" ref="H64" si="5">G64-J64-I64</f>
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <f>K64*Toolboxes!B$1+L64*Toolboxes!B$2+M64*Toolboxes!B$3+N64*Toolboxes!B$4+O64*Toolboxes!B$5</f>
+        <v>10</v>
+      </c>
+      <c r="O64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>194</v>
+      </c>
+      <c r="B65" t="s">
+        <v>189</v>
+      </c>
+      <c r="F65" t="s">
+        <v>43</v>
+      </c>
+      <c r="G65">
+        <v>10</v>
+      </c>
+      <c r="H65">
+        <f t="shared" ref="H65" si="6">G65-J65-I65</f>
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <f>K65*Toolboxes!B$1+L65*Toolboxes!B$2+M65*Toolboxes!B$3+N65*Toolboxes!B$4+O65*Toolboxes!B$5</f>
+        <v>10</v>
+      </c>
+      <c r="O65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>192</v>
+      </c>
+      <c r="B66" t="s">
+        <v>193</v>
+      </c>
+      <c r="F66" t="s">
+        <v>48</v>
+      </c>
+      <c r="G66">
+        <v>10</v>
+      </c>
+      <c r="H66">
+        <f>G66-J66-I66</f>
+        <v>0</v>
+      </c>
+      <c r="I66">
+        <f>K66*Toolboxes!B$1+L66*Toolboxes!B$2+M66*Toolboxes!B$3+N66*Toolboxes!B$4+O66*Toolboxes!B$5</f>
+        <v>10</v>
+      </c>
+      <c r="O66">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2663,27 +2906,32 @@
     <sortCondition ref="J1"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="H3:H59">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+  <conditionalFormatting sqref="H3:H66">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="7" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K3:N59">
-    <cfRule type="cellIs" dxfId="0" priority="7" operator="greaterThan">
+  <conditionalFormatting sqref="K3:O3 K4:N6 O4:O9 K8:N8 K10:O61">
+    <cfRule type="cellIs" dxfId="0" priority="8" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O63:O66">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="C7" r:id="rId1" display="https://www.bitsandparts.nl/Temperatuursensor-1-wire-Waterdicht-Dallas-DS18B20-2-meter-p109707" xr:uid="{9FFC9E7B-A3BC-41DC-9E4A-9E1829241AA9}"/>
+    <hyperlink ref="C8" r:id="rId1" display="https://www.bitsandparts.nl/Temperatuursensor-1-wire-Waterdicht-Dallas-DS18B20-2-meter-p109707" xr:uid="{9FFC9E7B-A3BC-41DC-9E4A-9E1829241AA9}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{A50BE7E1-47D7-462A-B893-02FD9AA08531}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2696,7 +2944,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87959254-01BC-824B-AB45-1EC51DD6A6CA}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -2709,7 +2957,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B2">
         <v>20</v>
@@ -2729,6 +2977,14 @@
       </c>
       <c r="B4">
         <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B5">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -2743,59 +2999,59 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" t="s">
         <v>173</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>174</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>175</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>176</v>
-      </c>
-      <c r="E2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F2" t="s">
-        <v>178</v>
-      </c>
-      <c r="G2" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C3" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H3" t="s">
         <v>180</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="G3" t="s">
-        <v>179</v>
-      </c>
-      <c r="H3" t="s">
-        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -2804,6 +3060,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c43a8398-59d6-4544-8889-d61e38456917">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="5290365f-c8d6-40d0-b44a-6be08a8a62f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004F5CB8A00F1A0841B3F9E89D33680BD0" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1c000b4385f70b7b1f84268cc1d8b6f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c43a8398-59d6-4544-8889-d61e38456917" xmlns:ns3="5290365f-c8d6-40d0-b44a-6be08a8a62f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dbeb20f29d81400e6a07d4788d4730" ns2:_="" ns3:_="">
     <xsd:import namespace="c43a8398-59d6-4544-8889-d61e38456917"/>
@@ -3058,27 +3334,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c43a8398-59d6-4544-8889-d61e38456917">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="5290365f-c8d6-40d0-b44a-6be08a8a62f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84604F91-3C59-4AE5-92E7-93618F763177}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17D6B607-A9B3-43F0-AF54-4344976BB527}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c43a8398-59d6-4544-8889-d61e38456917"/>
+    <ds:schemaRef ds:uri="5290365f-c8d6-40d0-b44a-6be08a8a62f3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED5F3FA2-F157-4A54-88A9-DA8FEABFC56D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3095,23 +3370,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17D6B607-A9B3-43F0-AF54-4344976BB527}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c43a8398-59d6-4544-8889-d61e38456917"/>
-    <ds:schemaRef ds:uri="5290365f-c8d6-40d0-b44a-6be08a8a62f3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84604F91-3C59-4AE5-92E7-93618F763177}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>